<commit_message>
Fix IMAGE() URLs to point to correct branch instead of main
The slide thumbnails exist on claude/sales-talking-points-90REn, not main.
Updated BASE_URL in generate_xlsx.py and regenerated thumbnails.csv and XLSX.

https://claude.ai/code/session_01JEWnefCUgvMjDtHk6Dib4y
</commit_message>
<xml_diff>
--- a/MOR_WPB_Sales_Talking_Points.xlsx
+++ b/MOR_WPB_Sales_Talking_Points.xlsx
@@ -491,7 +491,7 @@
     </row>
     <row r="2" ht="100" customHeight="1">
       <c r="A2" s="2">
-        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/main/slide-thumbnails/slide-01.jpg")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/claude/sales-talking-points-90REn/slide-thumbnails/slide-01.jpg")</f>
         <v/>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -522,7 +522,7 @@
     </row>
     <row r="3" ht="100" customHeight="1">
       <c r="A3" s="2">
-        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/main/slide-thumbnails/slide-02.jpg")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/claude/sales-talking-points-90REn/slide-thumbnails/slide-02.jpg")</f>
         <v/>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -553,7 +553,7 @@
     </row>
     <row r="4" ht="100" customHeight="1">
       <c r="A4" s="2">
-        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/main/slide-thumbnails/slide-03.jpg")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/claude/sales-talking-points-90REn/slide-thumbnails/slide-03.jpg")</f>
         <v/>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -584,7 +584,7 @@
     </row>
     <row r="5" ht="100" customHeight="1">
       <c r="A5" s="2">
-        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/main/slide-thumbnails/slide-04.jpg")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/claude/sales-talking-points-90REn/slide-thumbnails/slide-04.jpg")</f>
         <v/>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -615,7 +615,7 @@
     </row>
     <row r="6" ht="100" customHeight="1">
       <c r="A6" s="2">
-        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/main/slide-thumbnails/slide-05.jpg")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/claude/sales-talking-points-90REn/slide-thumbnails/slide-05.jpg")</f>
         <v/>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -646,7 +646,7 @@
     </row>
     <row r="7" ht="100" customHeight="1">
       <c r="A7" s="2">
-        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/main/slide-thumbnails/slide-06.jpg")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/claude/sales-talking-points-90REn/slide-thumbnails/slide-06.jpg")</f>
         <v/>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -677,7 +677,7 @@
     </row>
     <row r="8" ht="100" customHeight="1">
       <c r="A8" s="2">
-        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/main/slide-thumbnails/slide-07.jpg")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/claude/sales-talking-points-90REn/slide-thumbnails/slide-07.jpg")</f>
         <v/>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -708,7 +708,7 @@
     </row>
     <row r="9" ht="100" customHeight="1">
       <c r="A9" s="2">
-        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/main/slide-thumbnails/slide-08.jpg")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/claude/sales-talking-points-90REn/slide-thumbnails/slide-08.jpg")</f>
         <v/>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -739,7 +739,7 @@
     </row>
     <row r="10" ht="100" customHeight="1">
       <c r="A10" s="2">
-        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/main/slide-thumbnails/slide-09.jpg")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/claude/sales-talking-points-90REn/slide-thumbnails/slide-09.jpg")</f>
         <v/>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -770,7 +770,7 @@
     </row>
     <row r="11" ht="100" customHeight="1">
       <c r="A11" s="2">
-        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/main/slide-thumbnails/slide-10.jpg")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/claude/sales-talking-points-90REn/slide-thumbnails/slide-10.jpg")</f>
         <v/>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -801,7 +801,7 @@
     </row>
     <row r="12" ht="100" customHeight="1">
       <c r="A12" s="2">
-        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/main/slide-thumbnails/slide-11.jpg")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/claude/sales-talking-points-90REn/slide-thumbnails/slide-11.jpg")</f>
         <v/>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -832,7 +832,7 @@
     </row>
     <row r="13" ht="100" customHeight="1">
       <c r="A13" s="2">
-        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/main/slide-thumbnails/slide-12.jpg")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/claude/sales-talking-points-90REn/slide-thumbnails/slide-12.jpg")</f>
         <v/>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -863,7 +863,7 @@
     </row>
     <row r="14" ht="100" customHeight="1">
       <c r="A14" s="2">
-        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/main/slide-thumbnails/slide-13.jpg")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/claude/sales-talking-points-90REn/slide-thumbnails/slide-13.jpg")</f>
         <v/>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -894,7 +894,7 @@
     </row>
     <row r="15" ht="100" customHeight="1">
       <c r="A15" s="2">
-        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/main/slide-thumbnails/slide-14.jpg")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/claude/sales-talking-points-90REn/slide-thumbnails/slide-14.jpg")</f>
         <v/>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -925,7 +925,7 @@
     </row>
     <row r="16" ht="100" customHeight="1">
       <c r="A16" s="2">
-        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/main/slide-thumbnails/slide-15.jpg")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/claude/sales-talking-points-90REn/slide-thumbnails/slide-15.jpg")</f>
         <v/>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -956,7 +956,7 @@
     </row>
     <row r="17" ht="100" customHeight="1">
       <c r="A17" s="2">
-        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/main/slide-thumbnails/slide-16.jpg")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/claude/sales-talking-points-90REn/slide-thumbnails/slide-16.jpg")</f>
         <v/>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -987,7 +987,7 @@
     </row>
     <row r="18" ht="100" customHeight="1">
       <c r="A18" s="2">
-        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/main/slide-thumbnails/slide-17.jpg")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/claude/sales-talking-points-90REn/slide-thumbnails/slide-17.jpg")</f>
         <v/>
       </c>
       <c r="B18" s="3" t="inlineStr">
@@ -1018,7 +1018,7 @@
     </row>
     <row r="19" ht="100" customHeight="1">
       <c r="A19" s="2">
-        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/main/slide-thumbnails/slide-18.jpg")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/claude/sales-talking-points-90REn/slide-thumbnails/slide-18.jpg")</f>
         <v/>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -1049,7 +1049,7 @@
     </row>
     <row r="20" ht="100" customHeight="1">
       <c r="A20" s="2">
-        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/main/slide-thumbnails/slide-19.jpg")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/claude/sales-talking-points-90REn/slide-thumbnails/slide-19.jpg")</f>
         <v/>
       </c>
       <c r="B20" s="3" t="inlineStr">
@@ -1080,7 +1080,7 @@
     </row>
     <row r="21" ht="100" customHeight="1">
       <c r="A21" s="2">
-        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/main/slide-thumbnails/slide-20.jpg")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/claude/sales-talking-points-90REn/slide-thumbnails/slide-20.jpg")</f>
         <v/>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -1111,7 +1111,7 @@
     </row>
     <row r="22" ht="100" customHeight="1">
       <c r="A22" s="2">
-        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/main/slide-thumbnails/slide-21.jpg")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/claude/sales-talking-points-90REn/slide-thumbnails/slide-21.jpg")</f>
         <v/>
       </c>
       <c r="B22" s="3" t="inlineStr">
@@ -1147,7 +1147,7 @@
     </row>
     <row r="23" ht="100" customHeight="1">
       <c r="A23" s="2">
-        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/main/slide-thumbnails/slide-22.jpg")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/claude/sales-talking-points-90REn/slide-thumbnails/slide-22.jpg")</f>
         <v/>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -1178,7 +1178,7 @@
     </row>
     <row r="24" ht="100" customHeight="1">
       <c r="A24" s="2">
-        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/main/slide-thumbnails/slide-23.jpg")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/claude/sales-talking-points-90REn/slide-thumbnails/slide-23.jpg")</f>
         <v/>
       </c>
       <c r="B24" s="3" t="inlineStr">
@@ -1209,7 +1209,7 @@
     </row>
     <row r="25" ht="100" customHeight="1">
       <c r="A25" s="2">
-        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/main/slide-thumbnails/slide-24.jpg")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/claude/sales-talking-points-90REn/slide-thumbnails/slide-24.jpg")</f>
         <v/>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -1240,7 +1240,7 @@
     </row>
     <row r="26" ht="100" customHeight="1">
       <c r="A26" s="2">
-        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/main/slide-thumbnails/slide-25.jpg")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/claude/sales-talking-points-90REn/slide-thumbnails/slide-25.jpg")</f>
         <v/>
       </c>
       <c r="B26" s="3" t="inlineStr">
@@ -1271,7 +1271,7 @@
     </row>
     <row r="27" ht="100" customHeight="1">
       <c r="A27" s="2">
-        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/main/slide-thumbnails/slide-26.jpg")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/claude/sales-talking-points-90REn/slide-thumbnails/slide-26.jpg")</f>
         <v/>
       </c>
       <c r="B27" s="3" t="inlineStr">
@@ -1302,7 +1302,7 @@
     </row>
     <row r="28" ht="100" customHeight="1">
       <c r="A28" s="2">
-        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/main/slide-thumbnails/slide-27.jpg")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/claude/sales-talking-points-90REn/slide-thumbnails/slide-27.jpg")</f>
         <v/>
       </c>
       <c r="B28" s="3" t="inlineStr">
@@ -1333,7 +1333,7 @@
     </row>
     <row r="29" ht="100" customHeight="1">
       <c r="A29" s="2">
-        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/main/slide-thumbnails/slide-28.jpg")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/claude/sales-talking-points-90REn/slide-thumbnails/slide-28.jpg")</f>
         <v/>
       </c>
       <c r="B29" s="3" t="inlineStr">
@@ -1364,7 +1364,7 @@
     </row>
     <row r="30" ht="100" customHeight="1">
       <c r="A30" s="2">
-        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/main/slide-thumbnails/slide-29.jpg")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/claude/sales-talking-points-90REn/slide-thumbnails/slide-29.jpg")</f>
         <v/>
       </c>
       <c r="B30" s="3" t="inlineStr">
@@ -1391,7 +1391,7 @@
     </row>
     <row r="31" ht="100" customHeight="1">
       <c r="A31" s="2">
-        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/main/slide-thumbnails/slide-30.jpg")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/claude/sales-talking-points-90REn/slide-thumbnails/slide-30.jpg")</f>
         <v/>
       </c>
       <c r="B31" s="3" t="inlineStr">
@@ -1418,7 +1418,7 @@
     </row>
     <row r="32" ht="100" customHeight="1">
       <c r="A32" s="2">
-        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/main/slide-thumbnails/slide-31.jpg")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/claude/sales-talking-points-90REn/slide-thumbnails/slide-31.jpg")</f>
         <v/>
       </c>
       <c r="B32" s="3" t="inlineStr">
@@ -1445,7 +1445,7 @@
     </row>
     <row r="33" ht="100" customHeight="1">
       <c r="A33" s="2">
-        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/main/slide-thumbnails/slide-32.jpg")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/claude/sales-talking-points-90REn/slide-thumbnails/slide-32.jpg")</f>
         <v/>
       </c>
       <c r="B33" s="3" t="inlineStr">
@@ -1476,7 +1476,7 @@
     </row>
     <row r="34" ht="100" customHeight="1">
       <c r="A34" s="2">
-        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/main/slide-thumbnails/slide-33.jpg")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/claude/sales-talking-points-90REn/slide-thumbnails/slide-33.jpg")</f>
         <v/>
       </c>
       <c r="B34" s="3" t="inlineStr">
@@ -1507,7 +1507,7 @@
     </row>
     <row r="35" ht="100" customHeight="1">
       <c r="A35" s="2">
-        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/main/slide-thumbnails/slide-34.jpg")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/claude/sales-talking-points-90REn/slide-thumbnails/slide-34.jpg")</f>
         <v/>
       </c>
       <c r="B35" s="3" t="inlineStr">
@@ -1534,7 +1534,7 @@
     </row>
     <row r="36" ht="100" customHeight="1">
       <c r="A36" s="2">
-        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/main/slide-thumbnails/slide-35.jpg")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/claude/sales-talking-points-90REn/slide-thumbnails/slide-35.jpg")</f>
         <v/>
       </c>
       <c r="B36" s="3" t="inlineStr">
@@ -1565,7 +1565,7 @@
     </row>
     <row r="37" ht="100" customHeight="1">
       <c r="A37" s="2">
-        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/main/slide-thumbnails/slide-36.jpg")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/claude/sales-talking-points-90REn/slide-thumbnails/slide-36.jpg")</f>
         <v/>
       </c>
       <c r="B37" s="3" t="inlineStr">
@@ -1596,7 +1596,7 @@
     </row>
     <row r="38" ht="100" customHeight="1">
       <c r="A38" s="2">
-        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/main/slide-thumbnails/slide-37.jpg")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/claude/sales-talking-points-90REn/slide-thumbnails/slide-37.jpg")</f>
         <v/>
       </c>
       <c r="B38" s="3" t="inlineStr">
@@ -1627,7 +1627,7 @@
     </row>
     <row r="39" ht="100" customHeight="1">
       <c r="A39" s="2">
-        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/main/slide-thumbnails/slide-38.jpg")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/claude/sales-talking-points-90REn/slide-thumbnails/slide-38.jpg")</f>
         <v/>
       </c>
       <c r="B39" s="3" t="inlineStr">
@@ -1654,7 +1654,7 @@
     </row>
     <row r="40" ht="100" customHeight="1">
       <c r="A40" s="2">
-        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/main/slide-thumbnails/slide-39.jpg")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/claude/sales-talking-points-90REn/slide-thumbnails/slide-39.jpg")</f>
         <v/>
       </c>
       <c r="B40" s="3" t="inlineStr">
@@ -1681,7 +1681,7 @@
     </row>
     <row r="41" ht="100" customHeight="1">
       <c r="A41" s="2">
-        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/main/slide-thumbnails/slide-40.jpg")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/claude/sales-talking-points-90REn/slide-thumbnails/slide-40.jpg")</f>
         <v/>
       </c>
       <c r="B41" s="3" t="inlineStr">
@@ -1722,7 +1722,7 @@
     </row>
     <row r="42" ht="100" customHeight="1">
       <c r="A42" s="2">
-        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/main/slide-thumbnails/slide-41.jpg")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/claude/sales-talking-points-90REn/slide-thumbnails/slide-41.jpg")</f>
         <v/>
       </c>
       <c r="B42" s="3" t="inlineStr">
@@ -1753,7 +1753,7 @@
     </row>
     <row r="43" ht="100" customHeight="1">
       <c r="A43" s="2">
-        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/main/slide-thumbnails/slide-42.jpg")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/claude/sales-talking-points-90REn/slide-thumbnails/slide-42.jpg")</f>
         <v/>
       </c>
       <c r="B43" s="3" t="inlineStr">
@@ -1784,7 +1784,7 @@
     </row>
     <row r="44" ht="100" customHeight="1">
       <c r="A44" s="2">
-        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/main/slide-thumbnails/slide-43.jpg")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/CerveraDev/mor-wpb-workbook-tp/claude/sales-talking-points-90REn/slide-thumbnails/slide-43.jpg")</f>
         <v/>
       </c>
       <c r="B44" s="3" t="inlineStr">

</xml_diff>